<commit_message>
Cutting list: Width before Length, same as ModCraft
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MSSI-Cutting-List-Template.xlsx
+++ b/MSSI-Cutting-List-Template.xlsx
@@ -435,10 +435,10 @@
         <v>Qty</v>
       </c>
       <c r="F1" t="str">
+        <v>Width (mm)</v>
+      </c>
+      <c r="G1" t="str">
         <v>Length (mm)</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Width (mm)</v>
       </c>
       <c r="H1" t="str">
         <v>Edge Band</v>
@@ -473,10 +473,10 @@
         <v>2</v>
       </c>
       <c r="F2">
+        <v>560</v>
+      </c>
+      <c r="G2">
         <v>720</v>
-      </c>
-      <c r="G2">
-        <v>560</v>
       </c>
       <c r="H2" t="str">
         <v>1L 1S</v>
@@ -511,10 +511,10 @@
         <v>2</v>
       </c>
       <c r="F3">
+        <v>296</v>
+      </c>
+      <c r="G3">
         <v>716</v>
-      </c>
-      <c r="G3">
-        <v>296</v>
       </c>
       <c r="H3" t="str">
         <v>4S</v>
@@ -574,10 +574,10 @@
         <v>Faces</v>
       </c>
       <c r="D1" t="str">
+        <v>Width (mm)</v>
+      </c>
+      <c r="E1" t="str">
         <v>Length (mm)</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Width (mm)</v>
       </c>
       <c r="F1" t="str">
         <v>Qty</v>

</xml_diff>